<commit_message>
Remove min 1 identifier
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-br-core-medicationrequest.xlsx
+++ b/docs/StructureDefinition-br-core-medicationrequest.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-10T12:27:48-04:00</t>
+    <t>2026-09-10T13:05:34-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -3744,10 +3744,10 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="G11" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H11" t="s" s="2">
         <v>82</v>

</xml_diff>